<commit_message>
Fix team building: best-3 for Kickoff, China avoidance, team strength, Excel per-GW scoring
- Kickoff now uses best 3 games (was 2). Actual: 414 pts
- China players only used as budget fillers (0.1 expected) — no China in Kickoff team,
  minimal China in Santiago GW1 (NoMan as cheapest duelist filler, scored 1 pt)
- Team strength multiplier in Santiago expected pts: strong teams get 1.25x,
  weak teams 0.7x — favors players likely to advance
- Excel now shows per-GW actual points (was incorrectly showing all-GW best-2)
- Fixed Santiago optimizer: role-first phase fills mandatory slots before wildcards
- Santiago total: 295 pts (107 + 83 + 105)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VFL_2026_Kickoff_Pricing.xlsx
+++ b/VFL_2026_Kickoff_Pricing.xlsx
@@ -578,7 +578,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>31.2</v>
@@ -611,7 +611,7 @@
         <v>0.5</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>38.2</v>
@@ -644,7 +644,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>20.9</v>
@@ -677,7 +677,7 @@
         <v>-0.5</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>15.2</v>
@@ -710,7 +710,7 @@
         <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>35</v>
@@ -743,7 +743,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>25.6</v>
@@ -776,7 +776,7 @@
         <v>0.5</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>46</v>
@@ -809,7 +809,7 @@
         <v>-1</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>50.1</v>
@@ -842,7 +842,7 @@
         <v>-0.5</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>23.2</v>
@@ -875,7 +875,7 @@
         <v>1</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>14.2</v>
@@ -908,7 +908,7 @@
         <v>3.5</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>24.4</v>
@@ -941,7 +941,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>28.7</v>
@@ -974,7 +974,7 @@
         <v>-0.5</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>32.6</v>
@@ -1011,7 +1011,7 @@
         <v>4</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>41.9</v>
@@ -1044,7 +1044,7 @@
         <v>4.5</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>39.7</v>
@@ -1081,7 +1081,7 @@
         <v>-1</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>13.2</v>
@@ -1114,7 +1114,7 @@
         <v>2</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>10.8</v>
@@ -1147,7 +1147,7 @@
         <v>3.5</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>22.4</v>
@@ -1180,7 +1180,7 @@
         <v>1.5</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>45.8</v>
@@ -1213,7 +1213,7 @@
         <v>1.5</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>33.2</v>
@@ -1246,7 +1246,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>27.1</v>
@@ -1279,7 +1279,7 @@
         <v>1.5</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>38.9</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>11.3</v>
@@ -1345,7 +1345,7 @@
         <v>4.5</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>35.4</v>
@@ -1378,7 +1378,7 @@
         <v>3.5</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="H26" s="2" t="n">
         <v>23.8</v>
@@ -1411,7 +1411,7 @@
         <v>-2</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="H27" s="2" t="n">
         <v>16.1</v>
@@ -1444,7 +1444,7 @@
         <v>1</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H28" s="2" t="n">
         <v>29.5</v>
@@ -1477,7 +1477,7 @@
         <v>1</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>32.2</v>
@@ -1510,7 +1510,7 @@
         <v>2.5</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>42.7</v>
@@ -1543,7 +1543,7 @@
         <v>3.5</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="H31" s="2" t="n">
         <v>12.8</v>
@@ -1576,7 +1576,7 @@
         <v>2.5</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>20.5</v>
@@ -1609,7 +1609,7 @@
         <v>-2</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>3.3</v>
@@ -1642,7 +1642,7 @@
         <v>-2.5</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="H34" s="2" t="n">
         <v>6.6</v>
@@ -1675,7 +1675,7 @@
         <v>-2</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H35" s="2" t="n">
         <v>23.5</v>
@@ -1708,7 +1708,7 @@
         <v>-2</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>6.6</v>
@@ -1741,7 +1741,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>19.6</v>
@@ -1774,7 +1774,7 @@
         <v>2</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H38" s="2" t="n">
         <v>27.6</v>
@@ -1807,7 +1807,7 @@
         <v>0.5</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H39" s="2" t="n">
         <v>44.7</v>
@@ -1844,7 +1844,7 @@
         <v>4.5</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="H40" s="2" t="n">
         <v>36.9</v>
@@ -1881,7 +1881,7 @@
         <v>-3</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="H41" s="2" t="n">
         <v>2.9</v>
@@ -1914,7 +1914,7 @@
         <v>3.5</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H42" s="2" t="n">
         <v>25</v>
@@ -1947,7 +1947,7 @@
         <v>1</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H43" s="2" t="n">
         <v>41.9</v>
@@ -2013,7 +2013,7 @@
         <v>3.5</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H45" s="2" t="n">
         <v>25.9</v>
@@ -2050,7 +2050,7 @@
         <v>-1.5</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H46" s="2" t="n">
         <v>29.1</v>
@@ -2083,7 +2083,7 @@
         <v>-1</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H47" s="2" t="n">
         <v>23</v>
@@ -2116,7 +2116,7 @@
         <v>-1.5</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="H48" s="2" t="n">
         <v>5.9</v>
@@ -2149,7 +2149,7 @@
         <v>-1.5</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="H49" s="2" t="n">
         <v>12.2</v>
@@ -2182,7 +2182,7 @@
         <v>-2</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="H50" s="2" t="n">
         <v>18.6</v>
@@ -2215,7 +2215,7 @@
         <v>-0.5</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="H51" s="2" t="n">
         <v>23.1</v>
@@ -2248,7 +2248,7 @@
         <v>-1</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="H52" s="2" t="n">
         <v>10.4</v>
@@ -2281,7 +2281,7 @@
         <v>0</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H53" s="2" t="n">
         <v>17.7</v>
@@ -2318,7 +2318,7 @@
         <v>1</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="H54" s="2" t="n">
         <v>22.6</v>
@@ -2351,7 +2351,7 @@
         <v>1.5</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="H55" s="2" t="n">
         <v>10.2</v>
@@ -2384,7 +2384,7 @@
         <v>1.5</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="H56" s="2" t="n">
         <v>10.2</v>
@@ -2417,7 +2417,7 @@
         <v>0.5</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="H57" s="2" t="n">
         <v>20.9</v>
@@ -2450,7 +2450,7 @@
         <v>1</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="H58" s="2" t="n">
         <v>28.4</v>
@@ -2483,7 +2483,7 @@
         <v>1.5</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="H59" s="2" t="n">
         <v>22.1</v>
@@ -2520,7 +2520,7 @@
         <v>1.5</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="H60" s="2" t="n">
         <v>14.8</v>
@@ -2553,7 +2553,7 @@
         <v>1.5</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="H61" s="2" t="n">
         <v>18.3</v>
@@ -2586,7 +2586,7 @@
         <v>3</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="H62" s="2" t="n">
         <v>19.8</v>
@@ -2619,7 +2619,7 @@
         <v>2</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H63" s="2" t="n">
         <v>16.2</v>
@@ -2652,7 +2652,7 @@
         <v>3.5</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H64" s="2" t="n">
         <v>32.7</v>
@@ -2689,7 +2689,7 @@
         <v>-0.5</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H65" s="2" t="n">
         <v>13.8</v>
@@ -2722,7 +2722,7 @@
         <v>-1.5</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="H66" s="2" t="n">
         <v>4.1</v>
@@ -2755,7 +2755,7 @@
         <v>-0.5</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="H67" s="2" t="n">
         <v>17.7</v>
@@ -2792,7 +2792,7 @@
         <v>2</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H68" s="2" t="n">
         <v>8.800000000000001</v>
@@ -2825,7 +2825,7 @@
         <v>2</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H69" s="2" t="n">
         <v>5.5</v>
@@ -2858,7 +2858,7 @@
         <v>2</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H70" s="2" t="n">
         <v>11.7</v>
@@ -2895,7 +2895,7 @@
         <v>2.5</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>18.2</v>
@@ -2928,7 +2928,7 @@
         <v>3</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="H72" s="2" t="n">
         <v>43.4</v>
@@ -2961,7 +2961,7 @@
         <v>2</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="H73" s="2" t="n">
         <v>16.9</v>
@@ -2994,7 +2994,7 @@
         <v>1</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H74" s="2" t="n">
         <v>3</v>
@@ -3027,7 +3027,7 @@
         <v>1</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H75" s="2" t="n">
         <v>23.9</v>
@@ -3064,7 +3064,7 @@
         <v>0.5</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="H76" s="2" t="n">
         <v>4.3</v>
@@ -3097,7 +3097,7 @@
         <v>1.5</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="H77" s="2" t="n">
         <v>9.800000000000001</v>
@@ -3130,7 +3130,7 @@
         <v>-1</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="H78" s="2" t="n">
         <v>18.5</v>
@@ -3163,7 +3163,7 @@
         <v>-2</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H79" s="2" t="n">
         <v>4.8</v>
@@ -3196,7 +3196,7 @@
         <v>2.5</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H80" s="2" t="n">
         <v>9.800000000000001</v>
@@ -3233,7 +3233,7 @@
         <v>-4</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H81" s="2" t="n">
         <v>12.6</v>
@@ -3266,7 +3266,7 @@
         <v>-1.5</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H82" s="2" t="n">
         <v>3.4</v>
@@ -3299,7 +3299,7 @@
         <v>-2</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="H83" s="2" t="n">
         <v>6.7</v>
@@ -3332,7 +3332,7 @@
         <v>-1.5</v>
       </c>
       <c r="G84" s="2" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="H84" s="2" t="n">
         <v>12.3</v>
@@ -3369,7 +3369,7 @@
         <v>-1.5</v>
       </c>
       <c r="G85" s="2" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="H85" s="2" t="n">
         <v>14</v>
@@ -3402,7 +3402,7 @@
         <v>1.5</v>
       </c>
       <c r="G86" s="2" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H86" s="2" t="n">
         <v>15.9</v>
@@ -3476,7 +3476,7 @@
         <v>-1</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H88" s="2" t="n">
         <v>20.3</v>
@@ -3509,7 +3509,7 @@
         <v>-1.5</v>
       </c>
       <c r="G89" s="2" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="H89" s="2" t="n">
         <v>11.3</v>
@@ -3542,7 +3542,7 @@
         <v>3</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H90" s="2" t="n">
         <v>9.5</v>
@@ -3579,7 +3579,7 @@
         <v>1.5</v>
       </c>
       <c r="G91" s="2" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H91" s="2" t="n">
         <v>31.3</v>
@@ -3612,7 +3612,7 @@
         <v>1.5</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="H92" s="2" t="n">
         <v>9.300000000000001</v>
@@ -3645,7 +3645,7 @@
         <v>3.5</v>
       </c>
       <c r="G93" s="2" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H93" s="2" t="n">
         <v>0</v>
@@ -3682,7 +3682,7 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H94" s="2" t="n">
         <v>22.2</v>
@@ -3719,7 +3719,7 @@
         <v>1</v>
       </c>
       <c r="G95" s="2" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="H95" s="2" t="n">
         <v>5.1</v>
@@ -3756,7 +3756,7 @@
         <v>0.5</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="H96" s="2" t="n">
         <v>18.9</v>
@@ -3789,7 +3789,7 @@
         <v>-0.5</v>
       </c>
       <c r="G97" s="2" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="H97" s="2" t="n">
         <v>5</v>
@@ -3826,7 +3826,7 @@
         <v>0.5</v>
       </c>
       <c r="G98" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H98" s="2" t="n">
         <v>4.1</v>
@@ -3863,7 +3863,7 @@
         <v>-2</v>
       </c>
       <c r="G99" s="2" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H99" s="2" t="n">
         <v>1.7</v>
@@ -3900,7 +3900,7 @@
         <v>-1</v>
       </c>
       <c r="G100" s="2" t="n">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="H100" s="2" t="n">
         <v>8.4</v>
@@ -3937,7 +3937,7 @@
         <v>-0.5</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="H101" s="2" t="n">
         <v>17.9</v>
@@ -4007,7 +4007,7 @@
         <v>1</v>
       </c>
       <c r="G103" s="2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="H103" s="2" t="n">
         <v>10.5</v>
@@ -4040,7 +4040,7 @@
         <v>1</v>
       </c>
       <c r="G104" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H104" s="2" t="n">
         <v>14.3</v>
@@ -4077,7 +4077,7 @@
         <v>0</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H105" s="2" t="n">
         <v>11.6</v>
@@ -4114,7 +4114,7 @@
         <v>0</v>
       </c>
       <c r="G106" s="2" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H106" s="2" t="n">
         <v>13.8</v>
@@ -4147,7 +4147,7 @@
         <v>1</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="H107" s="2" t="n">
         <v>7.5</v>
@@ -4180,7 +4180,7 @@
         <v>0</v>
       </c>
       <c r="G108" s="2" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H108" s="2" t="n">
         <v>21.3</v>
@@ -4213,7 +4213,7 @@
         <v>-2</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H109" s="2" t="n">
         <v>4.5</v>
@@ -4246,7 +4246,7 @@
         <v>1.5</v>
       </c>
       <c r="G110" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H110" s="2" t="n">
         <v>10.7</v>
@@ -4279,7 +4279,7 @@
         <v>1</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="H111" s="2" t="n">
         <v>22.9</v>
@@ -4312,7 +4312,7 @@
         <v>0.5</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H112" s="2" t="n">
         <v>18.1</v>
@@ -4345,7 +4345,7 @@
         <v>-5</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="H113" s="2" t="n">
         <v>6.2</v>
@@ -4382,7 +4382,7 @@
         <v>1.5</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H114" s="2" t="n">
         <v>3.7</v>
@@ -4419,7 +4419,7 @@
         <v>0.5</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H115" s="2" t="n">
         <v>4</v>
@@ -4456,7 +4456,7 @@
         <v>0.5</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H116" s="2" t="n">
         <v>40.5</v>
@@ -4489,7 +4489,7 @@
         <v>-0.5</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="H117" s="2" t="n">
         <v>17</v>
@@ -4522,7 +4522,7 @@
         <v>0.5</v>
       </c>
       <c r="G118" s="2" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H118" s="2" t="n">
         <v>4.3</v>
@@ -4555,7 +4555,7 @@
         <v>2</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H119" s="2" t="n">
         <v>6.4</v>
@@ -4588,7 +4588,7 @@
         <v>0</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H120" s="2" t="n">
         <v>17.8</v>
@@ -4621,7 +4621,7 @@
         <v>-0.5</v>
       </c>
       <c r="G121" s="2" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="H121" s="2" t="n">
         <v>16.9</v>
@@ -4654,7 +4654,7 @@
         <v>-0.5</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="H122" s="2" t="n">
         <v>11.6</v>
@@ -4687,7 +4687,7 @@
         <v>-0.5</v>
       </c>
       <c r="G123" s="2" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="H123" s="2" t="n">
         <v>13</v>
@@ -4720,7 +4720,7 @@
         <v>1.5</v>
       </c>
       <c r="G124" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H124" s="2" t="n">
         <v>0.7</v>
@@ -4757,7 +4757,7 @@
         <v>1.5</v>
       </c>
       <c r="G125" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H125" s="2" t="n">
         <v>10.8</v>
@@ -4794,7 +4794,7 @@
         <v>2</v>
       </c>
       <c r="G126" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="H126" s="2" t="n">
         <v>5.3</v>
@@ -4831,7 +4831,7 @@
         <v>0</v>
       </c>
       <c r="G127" s="2" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="H127" s="2" t="n">
         <v>5.3</v>
@@ -4868,7 +4868,7 @@
         <v>1.5</v>
       </c>
       <c r="G128" s="2" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="H128" s="2" t="n">
         <v>0</v>
@@ -4905,7 +4905,7 @@
         <v>-1.5</v>
       </c>
       <c r="G129" s="2" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="H129" s="2" t="n">
         <v>5.4</v>
@@ -4942,7 +4942,7 @@
         <v>-2.5</v>
       </c>
       <c r="G130" s="2" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="H130" s="2" t="n">
         <v>7.8</v>
@@ -4975,7 +4975,7 @@
         <v>-1</v>
       </c>
       <c r="G131" s="2" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="H131" s="2" t="n">
         <v>12.3</v>
@@ -5012,7 +5012,7 @@
         <v>0.5</v>
       </c>
       <c r="G132" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H132" s="2" t="n">
         <v>3</v>
@@ -5049,7 +5049,7 @@
         <v>1</v>
       </c>
       <c r="G133" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H133" s="2" t="n">
         <v>2.2</v>
@@ -5086,7 +5086,7 @@
         <v>-0.5</v>
       </c>
       <c r="G134" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H134" s="2" t="n">
         <v>1</v>
@@ -5123,7 +5123,7 @@
         <v>-0.5</v>
       </c>
       <c r="G135" s="2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H135" s="2" t="n">
         <v>3.3</v>
@@ -5156,7 +5156,7 @@
         <v>-1</v>
       </c>
       <c r="G136" s="2" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H136" s="2" t="n">
         <v>8.1</v>
@@ -5189,7 +5189,7 @@
         <v>0.5</v>
       </c>
       <c r="G137" s="2" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="H137" s="2" t="n">
         <v>2</v>
@@ -5222,7 +5222,7 @@
         <v>0.5</v>
       </c>
       <c r="G138" s="2" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="H138" s="2" t="n">
         <v>11.2</v>
@@ -5255,7 +5255,7 @@
         <v>1.5</v>
       </c>
       <c r="G139" s="2" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="H139" s="2" t="n">
         <v>5.9</v>
@@ -5292,7 +5292,7 @@
         <v>0.5</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="H140" s="2" t="n">
         <v>8.9</v>
@@ -5325,7 +5325,7 @@
         <v>0.5</v>
       </c>
       <c r="G141" s="2" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="H141" s="2" t="n">
         <v>11.3</v>
@@ -5358,7 +5358,7 @@
         <v>-1.5</v>
       </c>
       <c r="G142" s="2" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H142" s="2" t="n">
         <v>2.8</v>
@@ -5395,7 +5395,7 @@
         <v>-1</v>
       </c>
       <c r="G143" s="2" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="H143" s="2" t="n">
         <v>6</v>
@@ -5428,7 +5428,7 @@
         <v>-4</v>
       </c>
       <c r="G144" s="2" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H144" s="2" t="n">
         <v>9.800000000000001</v>
@@ -5461,7 +5461,7 @@
         <v>0</v>
       </c>
       <c r="G145" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H145" s="2" t="n">
         <v>4.7</v>
@@ -5494,7 +5494,7 @@
         <v>0.5</v>
       </c>
       <c r="G146" s="2" t="n">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="H146" s="2" t="n">
         <v>9.1</v>
@@ -5531,7 +5531,7 @@
         <v>-2</v>
       </c>
       <c r="G147" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H147" s="2" t="n">
         <v>1.2</v>
@@ -5568,7 +5568,7 @@
         <v>-2</v>
       </c>
       <c r="G148" s="2" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H148" s="2" t="n">
         <v>0.5</v>
@@ -5605,7 +5605,7 @@
         <v>-4</v>
       </c>
       <c r="G149" s="2" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="H149" s="2" t="n">
         <v>2.9</v>
@@ -5642,7 +5642,7 @@
         <v>1</v>
       </c>
       <c r="G150" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H150" s="2" t="n">
         <v>8.699999999999999</v>
@@ -5679,7 +5679,7 @@
         <v>0.5</v>
       </c>
       <c r="G151" s="2" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="H151" s="2" t="n">
         <v>13</v>
@@ -5712,7 +5712,7 @@
         <v>-0.5</v>
       </c>
       <c r="G152" s="2" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="H152" s="2" t="n">
         <v>13.3</v>
@@ -5745,7 +5745,7 @@
         <v>-1</v>
       </c>
       <c r="G153" s="2" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="H153" s="2" t="n">
         <v>15.3</v>
@@ -5778,7 +5778,7 @@
         <v>0</v>
       </c>
       <c r="G154" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H154" s="2" t="n">
         <v>7.7</v>
@@ -5811,7 +5811,7 @@
         <v>0.5</v>
       </c>
       <c r="G155" s="2" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H155" s="2" t="n">
         <v>1.9</v>
@@ -5844,7 +5844,7 @@
         <v>0</v>
       </c>
       <c r="G156" s="2" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H156" s="2" t="n">
         <v>2.4</v>
@@ -5881,7 +5881,7 @@
         <v>-1.5</v>
       </c>
       <c r="G157" s="2" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="H157" s="2" t="n">
         <v>9.4</v>
@@ -5914,7 +5914,7 @@
         <v>-2.5</v>
       </c>
       <c r="G158" s="2" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="H158" s="2" t="n">
         <v>9.300000000000001</v>
@@ -5951,7 +5951,7 @@
         <v>-3.5</v>
       </c>
       <c r="G159" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H159" s="2" t="n">
         <v>6.5</v>
@@ -6021,7 +6021,7 @@
         <v>-1</v>
       </c>
       <c r="G161" s="2" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H161" s="2" t="n">
         <v>10.7</v>
@@ -6054,7 +6054,7 @@
         <v>-1</v>
       </c>
       <c r="G162" s="2" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H162" s="2" t="n">
         <v>24.8</v>
@@ -6091,7 +6091,7 @@
         <v>-1</v>
       </c>
       <c r="G163" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H163" s="2" t="n">
         <v>66.90000000000001</v>
@@ -6124,7 +6124,7 @@
         <v>-1.5</v>
       </c>
       <c r="G164" s="2" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="H164" s="2" t="n">
         <v>8.9</v>
@@ -6157,7 +6157,7 @@
         <v>-1.5</v>
       </c>
       <c r="G165" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H165" s="2" t="n">
         <v>2.7</v>
@@ -6194,7 +6194,7 @@
         <v>-0.5</v>
       </c>
       <c r="G166" s="2" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H166" s="2" t="n">
         <v>8.199999999999999</v>
@@ -6227,7 +6227,7 @@
         <v>-1.5</v>
       </c>
       <c r="G167" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H167" s="2" t="n">
         <v>3.7</v>
@@ -6301,7 +6301,7 @@
         <v>-5</v>
       </c>
       <c r="G169" s="2" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="H169" s="2" t="n">
         <v>11.6</v>
@@ -6375,7 +6375,7 @@
         <v>-4</v>
       </c>
       <c r="G171" s="2" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H171" s="2" t="n">
         <v>3.2</v>
@@ -6412,7 +6412,7 @@
         <v>-3.5</v>
       </c>
       <c r="G172" s="2" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="H172" s="2" t="n">
         <v>5</v>
@@ -6445,7 +6445,7 @@
         <v>-3</v>
       </c>
       <c r="G173" s="2" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H173" s="2" t="n">
         <v>4.2</v>
@@ -6478,7 +6478,7 @@
         <v>0</v>
       </c>
       <c r="G174" s="2" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H174" s="2" t="n">
         <v>60.6</v>
@@ -6544,7 +6544,7 @@
         <v>-3</v>
       </c>
       <c r="G176" s="2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="H176" s="2" t="n">
         <v>2.4</v>
@@ -6581,7 +6581,7 @@
         <v>-1.5</v>
       </c>
       <c r="G177" s="2" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H177" s="2" t="n">
         <v>6.1</v>
@@ -6618,7 +6618,7 @@
         <v>-1.5</v>
       </c>
       <c r="G178" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H178" s="2" t="n">
         <v>17.7</v>
@@ -6651,7 +6651,7 @@
         <v>-4.5</v>
       </c>
       <c r="G179" s="2" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="H179" s="2" t="n">
         <v>5.8</v>
@@ -6721,7 +6721,7 @@
         <v>0</v>
       </c>
       <c r="G181" s="2" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H181" s="2" t="n">
         <v>21.9</v>
@@ -6815,12 +6815,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>brawk</t>
+          <t>Kushy</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>NRG Esports</t>
+          <t>Rex Regum Qeon</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -6829,20 +6829,20 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>10.5</v>
+        <v>7.5</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>32.6</v>
+        <v>30.2</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Free1ng</t>
+          <t>MaKo</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -6852,125 +6852,125 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>26.2</v>
+        <v>35.7</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Francis</t>
+          <t>SociablEE</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Nongshim RedForce</t>
+          <t>Natus Vincere</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
         <v>8</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>24.7</v>
+        <v>34.1</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Kushy</t>
+          <t>Free1ng</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Rex Regum Qeon</t>
+          <t>DRX</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>22.4</v>
+        <v>34.9</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SociablEE</t>
+          <t>BABYBAY</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Natus Vincere</t>
+          <t>G2 Esports</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>S</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>25</v>
+        <v>35.6</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Ruxic</t>
+          <t>brawk</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Natus Vincere</t>
+          <t>NRG Esports</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>I</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>11.5</v>
+        <v>10.5</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>29.8</v>
+        <v>44</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -6994,7 +6994,7 @@
         <v>9.5</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>28.1</v>
+        <v>38.9</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>23</v>
@@ -7004,112 +7004,112 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Sato</t>
+          <t>JohnQT</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>LEVIATAN</t>
+          <t>Sentinels</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>14</v>
+        <v>7.5</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>36.2</v>
+        <v>28.7</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>IGL</t>
-        </is>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Cauanzin</t>
+          <t>PROFEK</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>LOUD</t>
+          <t>Team Vitality</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>6.5</v>
+        <v>9</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>18.4</v>
+        <v>32.8</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>JohnQT</t>
+          <t>Sato</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Sentinels</t>
+          <t>LEVIATAN</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>7.5</v>
+        <v>14</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>20.8</v>
+        <v>50.5</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
+        <v>26</v>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>IGL</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>BABYBAY</t>
+          <t>Francis</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>G2 Esports</t>
+          <t>Nongshim RedForce</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>24.6</v>
+        <v>33.2</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -7120,13 +7120,13 @@
         </is>
       </c>
       <c r="D14" s="9" t="n">
-        <v>100</v>
+        <v>99.5</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>324.8</v>
+        <v>449.2</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>291</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel fixes: Kickoff shows Best-3, Santiago shows per-GW Best-2 columns
- Kickoff Prices sheet: "Actual Best-3 Pts" (was Best-2)
- Santiago Prices sheet: 3 separate columns "Best-2 GW1/GW2/GW3" instead of 1
- Stronger tournament longevity bonus for GW1 team picks
- Relaxed role constraints on transfers (try same-role first, then any)
- More transfer attempts to handle failed swaps

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VFL_2026_Kickoff_Pricing.xlsx
+++ b/VFL_2026_Kickoff_Pricing.xlsx
@@ -538,7 +538,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Actual Best-2 Pts</t>
+          <t>Actual Best-3 Pts</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -6793,12 +6793,12 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>Expected Best-2</t>
+          <t>Expected Best-3</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Actual Best-2</t>
+          <t>Actual Best-3</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Add expected points display for Kickoff and Stage 1
- Compute bootstrap expected points for all players (not just team picks)
- Kickoff: show Expected vs Actual best-3 with correlation (0.373) and MAE (13.7)
- Stage 1: predict total points across 5 gameweeks using all data through Santiago
- Add Expected Pts column to Excel Prices sheets
- New Stage 1 Predictions Excel with per-player expected total points
- Refactor: extract compute_pool_expected_pts() for reuse across events

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VFL_2026_Kickoff_Pricing.xlsx
+++ b/VFL_2026_Kickoff_Pricing.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I181"/>
+  <dimension ref="A1:J181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -501,8 +501,9 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,15 +539,20 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Expected Pts</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Actual Best-3 Pts</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Pick%</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Uncertainty</t>
         </is>
@@ -578,12 +584,15 @@
         <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="I2" s="2" t="n">
         <v>31.2</v>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -611,12 +620,15 @@
         <v>0.5</v>
       </c>
       <c r="G3" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H3" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="I3" s="2" t="n">
         <v>38.2</v>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -644,12 +656,15 @@
         <v>0</v>
       </c>
       <c r="G4" s="2" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="I4" s="2" t="n">
         <v>20.9</v>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -677,12 +692,15 @@
         <v>-0.5</v>
       </c>
       <c r="G5" s="2" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="I5" s="2" t="n">
         <v>15.2</v>
       </c>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -710,12 +728,15 @@
         <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="H6" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="I6" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -743,12 +764,15 @@
         <v>0</v>
       </c>
       <c r="G7" s="2" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="H7" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="I7" s="2" t="n">
         <v>25.6</v>
       </c>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -776,12 +800,15 @@
         <v>0.5</v>
       </c>
       <c r="G8" s="2" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="I8" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -809,12 +836,15 @@
         <v>-1</v>
       </c>
       <c r="G9" s="2" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="H9" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="I9" s="2" t="n">
         <v>50.1</v>
       </c>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -842,12 +872,15 @@
         <v>-0.5</v>
       </c>
       <c r="G10" s="2" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="H10" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="I10" s="2" t="n">
         <v>23.2</v>
       </c>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -875,12 +908,15 @@
         <v>1</v>
       </c>
       <c r="G11" s="2" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="H11" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="I11" s="2" t="n">
         <v>14.2</v>
       </c>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -908,12 +944,15 @@
         <v>3.5</v>
       </c>
       <c r="G12" s="2" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="H12" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="I12" s="2" t="n">
         <v>24.4</v>
       </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -941,12 +980,15 @@
         <v>0</v>
       </c>
       <c r="G13" s="2" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="H13" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="I13" s="2" t="n">
         <v>28.7</v>
       </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -974,12 +1016,15 @@
         <v>-0.5</v>
       </c>
       <c r="G14" s="2" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="H14" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="I14" s="2" t="n">
         <v>32.6</v>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -1011,12 +1056,15 @@
         <v>4</v>
       </c>
       <c r="G15" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="H15" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="I15" s="2" t="n">
         <v>41.9</v>
       </c>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1044,12 +1092,15 @@
         <v>4.5</v>
       </c>
       <c r="G16" s="2" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="H16" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="I16" s="2" t="n">
         <v>39.7</v>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -1081,12 +1132,15 @@
         <v>-1</v>
       </c>
       <c r="G17" s="2" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="H17" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="I17" s="2" t="n">
         <v>13.2</v>
       </c>
-      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1114,12 +1168,15 @@
         <v>2</v>
       </c>
       <c r="G18" s="2" t="n">
+        <v>35.1</v>
+      </c>
+      <c r="H18" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="I18" s="2" t="n">
         <v>10.8</v>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1147,12 +1204,15 @@
         <v>3.5</v>
       </c>
       <c r="G19" s="2" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="H19" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="I19" s="2" t="n">
         <v>22.4</v>
       </c>
-      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1180,12 +1240,15 @@
         <v>1.5</v>
       </c>
       <c r="G20" s="2" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="H20" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="I20" s="2" t="n">
         <v>45.8</v>
       </c>
-      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1213,12 +1276,15 @@
         <v>1.5</v>
       </c>
       <c r="G21" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H21" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="I21" s="2" t="n">
         <v>33.2</v>
       </c>
-      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1246,12 +1312,15 @@
         <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="H22" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="H22" s="2" t="n">
+      <c r="I22" s="2" t="n">
         <v>27.1</v>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1279,12 +1348,15 @@
         <v>1.5</v>
       </c>
       <c r="G23" s="2" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="H23" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="I23" s="2" t="n">
         <v>38.9</v>
       </c>
-      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1312,12 +1384,15 @@
         <v>-1</v>
       </c>
       <c r="G24" s="2" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="H24" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="I24" s="2" t="n">
         <v>11.3</v>
       </c>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1345,12 +1420,15 @@
         <v>4.5</v>
       </c>
       <c r="G25" s="2" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="H25" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="H25" s="2" t="n">
+      <c r="I25" s="2" t="n">
         <v>35.4</v>
       </c>
-      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1378,12 +1456,15 @@
         <v>3.5</v>
       </c>
       <c r="G26" s="2" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="H26" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="I26" s="2" t="n">
         <v>23.8</v>
       </c>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1411,12 +1492,15 @@
         <v>-2</v>
       </c>
       <c r="G27" s="2" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="H27" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="H27" s="2" t="n">
+      <c r="I27" s="2" t="n">
         <v>16.1</v>
       </c>
-      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1444,12 +1528,15 @@
         <v>1</v>
       </c>
       <c r="G28" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H28" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="I28" s="2" t="n">
         <v>29.5</v>
       </c>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1477,12 +1564,15 @@
         <v>1</v>
       </c>
       <c r="G29" s="2" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="H29" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="H29" s="2" t="n">
+      <c r="I29" s="2" t="n">
         <v>32.2</v>
       </c>
-      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1510,12 +1600,15 @@
         <v>2.5</v>
       </c>
       <c r="G30" s="2" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="H30" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="I30" s="2" t="n">
         <v>42.7</v>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1543,12 +1636,15 @@
         <v>3.5</v>
       </c>
       <c r="G31" s="2" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="H31" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="H31" s="2" t="n">
+      <c r="I31" s="2" t="n">
         <v>12.8</v>
       </c>
-      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1576,12 +1672,15 @@
         <v>2.5</v>
       </c>
       <c r="G32" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="H32" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="H32" s="2" t="n">
+      <c r="I32" s="2" t="n">
         <v>20.5</v>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1609,12 +1708,15 @@
         <v>-2</v>
       </c>
       <c r="G33" s="2" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H33" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="I33" s="2" t="n">
         <v>3.3</v>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1642,12 +1744,15 @@
         <v>-2.5</v>
       </c>
       <c r="G34" s="2" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="H34" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="H34" s="2" t="n">
+      <c r="I34" s="2" t="n">
         <v>6.6</v>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1675,12 +1780,15 @@
         <v>-2</v>
       </c>
       <c r="G35" s="2" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="H35" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H35" s="2" t="n">
+      <c r="I35" s="2" t="n">
         <v>23.5</v>
       </c>
-      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1708,12 +1816,15 @@
         <v>-2</v>
       </c>
       <c r="G36" s="2" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="H36" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H36" s="2" t="n">
+      <c r="I36" s="2" t="n">
         <v>6.6</v>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1741,12 +1852,15 @@
         <v>0</v>
       </c>
       <c r="G37" s="2" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="H37" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="I37" s="2" t="n">
         <v>19.6</v>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1774,12 +1888,15 @@
         <v>2</v>
       </c>
       <c r="G38" s="2" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="H38" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="I38" s="2" t="n">
         <v>27.6</v>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1807,12 +1924,15 @@
         <v>0.5</v>
       </c>
       <c r="G39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="I39" s="2" t="n">
         <v>44.7</v>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -1844,12 +1964,15 @@
         <v>4.5</v>
       </c>
       <c r="G40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="H40" s="2" t="n">
+      <c r="I40" s="2" t="n">
         <v>36.9</v>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -1881,12 +2004,15 @@
         <v>-3</v>
       </c>
       <c r="G41" s="2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H41" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="H41" s="2" t="n">
+      <c r="I41" s="2" t="n">
         <v>2.9</v>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1914,12 +2040,15 @@
         <v>3.5</v>
       </c>
       <c r="G42" s="2" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="H42" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="H42" s="2" t="n">
+      <c r="I42" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1947,12 +2076,15 @@
         <v>1</v>
       </c>
       <c r="G43" s="2" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="H43" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H43" s="2" t="n">
+      <c r="I43" s="2" t="n">
         <v>41.9</v>
       </c>
-      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1980,12 +2112,15 @@
         <v>1.5</v>
       </c>
       <c r="G44" s="2" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="H44" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="2" t="n">
+      <c r="I44" s="2" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2013,12 +2148,15 @@
         <v>3.5</v>
       </c>
       <c r="G45" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="H45" s="2" t="n">
+      <c r="I45" s="2" t="n">
         <v>25.9</v>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -2050,12 +2188,15 @@
         <v>-1.5</v>
       </c>
       <c r="G46" s="2" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="H46" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="H46" s="2" t="n">
+      <c r="I46" s="2" t="n">
         <v>29.1</v>
       </c>
-      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2083,12 +2224,15 @@
         <v>-1</v>
       </c>
       <c r="G47" s="2" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="H47" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H47" s="2" t="n">
+      <c r="I47" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2116,12 +2260,15 @@
         <v>-1.5</v>
       </c>
       <c r="G48" s="2" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="H48" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="H48" s="2" t="n">
+      <c r="I48" s="2" t="n">
         <v>5.9</v>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2149,12 +2296,15 @@
         <v>-1.5</v>
       </c>
       <c r="G49" s="2" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="H49" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="H49" s="2" t="n">
+      <c r="I49" s="2" t="n">
         <v>12.2</v>
       </c>
-      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2182,12 +2332,15 @@
         <v>-2</v>
       </c>
       <c r="G50" s="2" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="H50" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="I50" s="2" t="n">
         <v>18.6</v>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2215,12 +2368,15 @@
         <v>-0.5</v>
       </c>
       <c r="G51" s="2" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="H51" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H51" s="2" t="n">
+      <c r="I51" s="2" t="n">
         <v>23.1</v>
       </c>
-      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2248,12 +2404,15 @@
         <v>-1</v>
       </c>
       <c r="G52" s="2" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="H52" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="H52" s="2" t="n">
+      <c r="I52" s="2" t="n">
         <v>10.4</v>
       </c>
-      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2281,12 +2440,15 @@
         <v>0</v>
       </c>
       <c r="G53" s="2" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="H53" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H53" s="2" t="n">
+      <c r="I53" s="2" t="n">
         <v>17.7</v>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="J53" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -2318,12 +2480,15 @@
         <v>1</v>
       </c>
       <c r="G54" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="H54" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H54" s="2" t="n">
+      <c r="I54" s="2" t="n">
         <v>22.6</v>
       </c>
-      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2351,12 +2516,15 @@
         <v>1.5</v>
       </c>
       <c r="G55" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H55" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="H55" s="2" t="n">
+      <c r="I55" s="2" t="n">
         <v>10.2</v>
       </c>
-      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2384,12 +2552,15 @@
         <v>1.5</v>
       </c>
       <c r="G56" s="2" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="H56" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H56" s="2" t="n">
+      <c r="I56" s="2" t="n">
         <v>10.2</v>
       </c>
-      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2417,12 +2588,15 @@
         <v>0.5</v>
       </c>
       <c r="G57" s="2" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="H57" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="H57" s="2" t="n">
+      <c r="I57" s="2" t="n">
         <v>20.9</v>
       </c>
-      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2450,12 +2624,15 @@
         <v>1</v>
       </c>
       <c r="G58" s="2" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="H58" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H58" s="2" t="n">
+      <c r="I58" s="2" t="n">
         <v>28.4</v>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2483,12 +2660,15 @@
         <v>1.5</v>
       </c>
       <c r="G59" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="H59" s="2" t="n">
+      <c r="I59" s="2" t="n">
         <v>22.1</v>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="J59" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -2520,12 +2700,15 @@
         <v>1.5</v>
       </c>
       <c r="G60" s="2" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="H60" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H60" s="2" t="n">
+      <c r="I60" s="2" t="n">
         <v>14.8</v>
       </c>
-      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2553,12 +2736,15 @@
         <v>1.5</v>
       </c>
       <c r="G61" s="2" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="H61" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="H61" s="2" t="n">
+      <c r="I61" s="2" t="n">
         <v>18.3</v>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2586,12 +2772,15 @@
         <v>3</v>
       </c>
       <c r="G62" s="2" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="H62" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="H62" s="2" t="n">
+      <c r="I62" s="2" t="n">
         <v>19.8</v>
       </c>
-      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2619,12 +2808,15 @@
         <v>2</v>
       </c>
       <c r="G63" s="2" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="H63" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H63" s="2" t="n">
+      <c r="I63" s="2" t="n">
         <v>16.2</v>
       </c>
-      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2652,12 +2844,15 @@
         <v>3.5</v>
       </c>
       <c r="G64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="H64" s="2" t="n">
+      <c r="I64" s="2" t="n">
         <v>32.7</v>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="J64" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -2689,12 +2884,15 @@
         <v>-0.5</v>
       </c>
       <c r="G65" s="2" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="H65" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H65" s="2" t="n">
+      <c r="I65" s="2" t="n">
         <v>13.8</v>
       </c>
-      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2722,12 +2920,15 @@
         <v>-1.5</v>
       </c>
       <c r="G66" s="2" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="H66" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="H66" s="2" t="n">
+      <c r="I66" s="2" t="n">
         <v>4.1</v>
       </c>
-      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2755,12 +2956,15 @@
         <v>-0.5</v>
       </c>
       <c r="G67" s="2" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="H67" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="H67" s="2" t="n">
+      <c r="I67" s="2" t="n">
         <v>17.7</v>
       </c>
-      <c r="I67" s="2" t="inlineStr">
+      <c r="J67" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -2792,12 +2996,15 @@
         <v>2</v>
       </c>
       <c r="G68" s="2" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="H68" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="H68" s="2" t="n">
+      <c r="I68" s="2" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2825,12 +3032,15 @@
         <v>2</v>
       </c>
       <c r="G69" s="2" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="H69" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="H69" s="2" t="n">
+      <c r="I69" s="2" t="n">
         <v>5.5</v>
       </c>
-      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2858,12 +3068,15 @@
         <v>2</v>
       </c>
       <c r="G70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="H70" s="2" t="n">
+      <c r="I70" s="2" t="n">
         <v>11.7</v>
       </c>
-      <c r="I70" s="2" t="inlineStr">
+      <c r="J70" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -2895,12 +3108,15 @@
         <v>2.5</v>
       </c>
       <c r="G71" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H71" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H71" s="2" t="n">
+      <c r="I71" s="2" t="n">
         <v>18.2</v>
       </c>
-      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2928,12 +3144,15 @@
         <v>3</v>
       </c>
       <c r="G72" s="2" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="H72" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H72" s="2" t="n">
+      <c r="I72" s="2" t="n">
         <v>43.4</v>
       </c>
-      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2961,12 +3180,15 @@
         <v>2</v>
       </c>
       <c r="G73" s="2" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="H73" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="H73" s="2" t="n">
+      <c r="I73" s="2" t="n">
         <v>16.9</v>
       </c>
-      <c r="I73" s="2" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2994,12 +3216,15 @@
         <v>1</v>
       </c>
       <c r="G74" s="2" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="H74" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="H74" s="2" t="n">
+      <c r="I74" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3027,12 +3252,15 @@
         <v>1</v>
       </c>
       <c r="G75" s="2" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="H75" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H75" s="2" t="n">
+      <c r="I75" s="2" t="n">
         <v>23.9</v>
       </c>
-      <c r="I75" s="2" t="inlineStr">
+      <c r="J75" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -3064,12 +3292,15 @@
         <v>0.5</v>
       </c>
       <c r="G76" s="2" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="H76" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="H76" s="2" t="n">
+      <c r="I76" s="2" t="n">
         <v>4.3</v>
       </c>
-      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3097,12 +3328,15 @@
         <v>1.5</v>
       </c>
       <c r="G77" s="2" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="H77" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H77" s="2" t="n">
+      <c r="I77" s="2" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3130,12 +3364,15 @@
         <v>-1</v>
       </c>
       <c r="G78" s="2" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="H78" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="H78" s="2" t="n">
+      <c r="I78" s="2" t="n">
         <v>18.5</v>
       </c>
-      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3163,12 +3400,15 @@
         <v>-2</v>
       </c>
       <c r="G79" s="2" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="H79" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="H79" s="2" t="n">
+      <c r="I79" s="2" t="n">
         <v>4.8</v>
       </c>
-      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3196,12 +3436,15 @@
         <v>2.5</v>
       </c>
       <c r="G80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H80" s="2" t="n">
+      <c r="I80" s="2" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="I80" s="2" t="inlineStr">
+      <c r="J80" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3233,12 +3476,15 @@
         <v>-4</v>
       </c>
       <c r="G81" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="H81" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="H81" s="2" t="n">
+      <c r="I81" s="2" t="n">
         <v>12.6</v>
       </c>
-      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3266,12 +3512,15 @@
         <v>-1.5</v>
       </c>
       <c r="G82" s="2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H82" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H82" s="2" t="n">
+      <c r="I82" s="2" t="n">
         <v>3.4</v>
       </c>
-      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3299,12 +3548,15 @@
         <v>-2</v>
       </c>
       <c r="G83" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H83" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="H83" s="2" t="n">
+      <c r="I83" s="2" t="n">
         <v>6.7</v>
       </c>
-      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3332,12 +3584,15 @@
         <v>-1.5</v>
       </c>
       <c r="G84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="H84" s="2" t="n">
+      <c r="I84" s="2" t="n">
         <v>12.3</v>
       </c>
-      <c r="I84" s="2" t="inlineStr">
+      <c r="J84" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3369,12 +3624,15 @@
         <v>-1.5</v>
       </c>
       <c r="G85" s="2" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="H85" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H85" s="2" t="n">
+      <c r="I85" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3402,12 +3660,15 @@
         <v>1.5</v>
       </c>
       <c r="G86" s="2" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="H86" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H86" s="2" t="n">
+      <c r="I86" s="2" t="n">
         <v>15.9</v>
       </c>
-      <c r="I86" s="2" t="inlineStr">
+      <c r="J86" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -3439,12 +3700,15 @@
         <v>4</v>
       </c>
       <c r="G87" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H87" s="2" t="n">
+      <c r="I87" s="2" t="n">
         <v>14.3</v>
       </c>
-      <c r="I87" s="2" t="inlineStr">
+      <c r="J87" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3476,12 +3740,15 @@
         <v>-1</v>
       </c>
       <c r="G88" s="2" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="H88" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="H88" s="2" t="n">
+      <c r="I88" s="2" t="n">
         <v>20.3</v>
       </c>
-      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3509,12 +3776,15 @@
         <v>-1.5</v>
       </c>
       <c r="G89" s="2" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="H89" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="H89" s="2" t="n">
+      <c r="I89" s="2" t="n">
         <v>11.3</v>
       </c>
-      <c r="I89" s="2" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3542,12 +3812,15 @@
         <v>3</v>
       </c>
       <c r="G90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H90" s="2" t="n">
+      <c r="I90" s="2" t="n">
         <v>9.5</v>
       </c>
-      <c r="I90" s="2" t="inlineStr">
+      <c r="J90" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3579,12 +3852,15 @@
         <v>1.5</v>
       </c>
       <c r="G91" s="2" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="H91" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H91" s="2" t="n">
+      <c r="I91" s="2" t="n">
         <v>31.3</v>
       </c>
-      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3612,12 +3888,15 @@
         <v>1.5</v>
       </c>
       <c r="G92" s="2" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="H92" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H92" s="2" t="n">
+      <c r="I92" s="2" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3645,12 +3924,15 @@
         <v>3.5</v>
       </c>
       <c r="G93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="H93" s="2" t="n">
+      <c r="I93" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I93" s="2" t="inlineStr">
+      <c r="J93" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3682,12 +3964,15 @@
         <v>0.5</v>
       </c>
       <c r="G94" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H94" s="2" t="n">
+      <c r="I94" s="2" t="n">
         <v>22.2</v>
       </c>
-      <c r="I94" s="2" t="inlineStr">
+      <c r="J94" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3719,12 +4004,15 @@
         <v>1</v>
       </c>
       <c r="G95" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="H95" s="2" t="n">
+      <c r="I95" s="2" t="n">
         <v>5.1</v>
       </c>
-      <c r="I95" s="2" t="inlineStr">
+      <c r="J95" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3756,12 +4044,15 @@
         <v>0.5</v>
       </c>
       <c r="G96" s="2" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="H96" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="H96" s="2" t="n">
+      <c r="I96" s="2" t="n">
         <v>18.9</v>
       </c>
-      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3789,12 +4080,15 @@
         <v>-0.5</v>
       </c>
       <c r="G97" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="H97" s="2" t="n">
+      <c r="I97" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I97" s="2" t="inlineStr">
+      <c r="J97" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3826,12 +4120,15 @@
         <v>0.5</v>
       </c>
       <c r="G98" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H98" s="2" t="n">
+      <c r="I98" s="2" t="n">
         <v>4.1</v>
       </c>
-      <c r="I98" s="2" t="inlineStr">
+      <c r="J98" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3863,12 +4160,15 @@
         <v>-2</v>
       </c>
       <c r="G99" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H99" s="2" t="n">
+      <c r="I99" s="2" t="n">
         <v>1.7</v>
       </c>
-      <c r="I99" s="2" t="inlineStr">
+      <c r="J99" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3900,12 +4200,15 @@
         <v>-1</v>
       </c>
       <c r="G100" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="H100" s="2" t="n">
+      <c r="I100" s="2" t="n">
         <v>8.4</v>
       </c>
-      <c r="I100" s="2" t="inlineStr">
+      <c r="J100" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -3937,12 +4240,15 @@
         <v>-0.5</v>
       </c>
       <c r="G101" s="2" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="H101" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="H101" s="2" t="n">
+      <c r="I101" s="2" t="n">
         <v>17.9</v>
       </c>
-      <c r="I101" s="2" t="inlineStr">
+      <c r="J101" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -3974,12 +4280,15 @@
         <v>3.5</v>
       </c>
       <c r="G102" s="2" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="H102" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="H102" s="2" t="n">
+      <c r="I102" s="2" t="n">
         <v>32.9</v>
       </c>
-      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4007,12 +4316,15 @@
         <v>1</v>
       </c>
       <c r="G103" s="2" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="H103" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="H103" s="2" t="n">
+      <c r="I103" s="2" t="n">
         <v>10.5</v>
       </c>
-      <c r="I103" s="2" t="inlineStr"/>
+      <c r="J103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -4040,12 +4352,15 @@
         <v>1</v>
       </c>
       <c r="G104" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="H104" s="2" t="n">
+      <c r="I104" s="2" t="n">
         <v>14.3</v>
       </c>
-      <c r="I104" s="2" t="inlineStr">
+      <c r="J104" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -4077,12 +4392,15 @@
         <v>0</v>
       </c>
       <c r="G105" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="H105" s="2" t="n">
+      <c r="I105" s="2" t="n">
         <v>11.6</v>
       </c>
-      <c r="I105" s="2" t="inlineStr">
+      <c r="J105" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -4114,12 +4432,15 @@
         <v>0</v>
       </c>
       <c r="G106" s="2" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="H106" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H106" s="2" t="n">
+      <c r="I106" s="2" t="n">
         <v>13.8</v>
       </c>
-      <c r="I106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4147,12 +4468,15 @@
         <v>1</v>
       </c>
       <c r="G107" s="2" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="H107" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H107" s="2" t="n">
+      <c r="I107" s="2" t="n">
         <v>7.5</v>
       </c>
-      <c r="I107" s="2" t="inlineStr"/>
+      <c r="J107" s="2" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4180,12 +4504,15 @@
         <v>0</v>
       </c>
       <c r="G108" s="2" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="H108" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H108" s="2" t="n">
+      <c r="I108" s="2" t="n">
         <v>21.3</v>
       </c>
-      <c r="I108" s="2" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -4213,12 +4540,15 @@
         <v>-2</v>
       </c>
       <c r="G109" s="2" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="H109" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="H109" s="2" t="n">
+      <c r="I109" s="2" t="n">
         <v>4.5</v>
       </c>
-      <c r="I109" s="2" t="inlineStr"/>
+      <c r="J109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4246,12 +4576,15 @@
         <v>1.5</v>
       </c>
       <c r="G110" s="2" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="H110" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H110" s="2" t="n">
+      <c r="I110" s="2" t="n">
         <v>10.7</v>
       </c>
-      <c r="I110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4279,12 +4612,15 @@
         <v>1</v>
       </c>
       <c r="G111" s="2" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="H111" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H111" s="2" t="n">
+      <c r="I111" s="2" t="n">
         <v>22.9</v>
       </c>
-      <c r="I111" s="2" t="inlineStr"/>
+      <c r="J111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4312,12 +4648,15 @@
         <v>0.5</v>
       </c>
       <c r="G112" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H112" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H112" s="2" t="n">
+      <c r="I112" s="2" t="n">
         <v>18.1</v>
       </c>
-      <c r="I112" s="2" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4345,12 +4684,15 @@
         <v>-5</v>
       </c>
       <c r="G113" s="2" t="n">
+        <v>30.4</v>
+      </c>
+      <c r="H113" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H113" s="2" t="n">
+      <c r="I113" s="2" t="n">
         <v>6.2</v>
       </c>
-      <c r="I113" s="2" t="inlineStr">
+      <c r="J113" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -4382,12 +4724,15 @@
         <v>1.5</v>
       </c>
       <c r="G114" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="H114" s="2" t="n">
+      <c r="I114" s="2" t="n">
         <v>3.7</v>
       </c>
-      <c r="I114" s="2" t="inlineStr">
+      <c r="J114" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -4419,12 +4764,15 @@
         <v>0.5</v>
       </c>
       <c r="G115" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="H115" s="2" t="n">
+      <c r="I115" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="I115" s="2" t="inlineStr">
+      <c r="J115" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -4456,12 +4804,15 @@
         <v>0.5</v>
       </c>
       <c r="G116" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H116" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="H116" s="2" t="n">
+      <c r="I116" s="2" t="n">
         <v>40.5</v>
       </c>
-      <c r="I116" s="2" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -4489,12 +4840,15 @@
         <v>-0.5</v>
       </c>
       <c r="G117" s="2" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="H117" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H117" s="2" t="n">
+      <c r="I117" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="I117" s="2" t="inlineStr"/>
+      <c r="J117" s="2" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -4522,12 +4876,15 @@
         <v>0.5</v>
       </c>
       <c r="G118" s="2" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="H118" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H118" s="2" t="n">
+      <c r="I118" s="2" t="n">
         <v>4.3</v>
       </c>
-      <c r="I118" s="2" t="inlineStr"/>
+      <c r="J118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -4555,12 +4912,15 @@
         <v>2</v>
       </c>
       <c r="G119" s="2" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="H119" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H119" s="2" t="n">
+      <c r="I119" s="2" t="n">
         <v>6.4</v>
       </c>
-      <c r="I119" s="2" t="inlineStr"/>
+      <c r="J119" s="2" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -4588,12 +4948,15 @@
         <v>0</v>
       </c>
       <c r="G120" s="2" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="H120" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H120" s="2" t="n">
+      <c r="I120" s="2" t="n">
         <v>17.8</v>
       </c>
-      <c r="I120" s="2" t="inlineStr"/>
+      <c r="J120" s="2" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -4621,12 +4984,15 @@
         <v>-0.5</v>
       </c>
       <c r="G121" s="2" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="H121" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="H121" s="2" t="n">
+      <c r="I121" s="2" t="n">
         <v>16.9</v>
       </c>
-      <c r="I121" s="2" t="inlineStr"/>
+      <c r="J121" s="2" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -4654,12 +5020,15 @@
         <v>-0.5</v>
       </c>
       <c r="G122" s="2" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H122" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H122" s="2" t="n">
+      <c r="I122" s="2" t="n">
         <v>11.6</v>
       </c>
-      <c r="I122" s="2" t="inlineStr"/>
+      <c r="J122" s="2" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -4687,12 +5056,15 @@
         <v>-0.5</v>
       </c>
       <c r="G123" s="2" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="H123" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="H123" s="2" t="n">
+      <c r="I123" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="I123" s="2" t="inlineStr"/>
+      <c r="J123" s="2" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -4720,12 +5092,15 @@
         <v>1.5</v>
       </c>
       <c r="G124" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H124" s="2" t="n">
+      <c r="I124" s="2" t="n">
         <v>0.7</v>
       </c>
-      <c r="I124" s="2" t="inlineStr">
+      <c r="J124" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -4757,12 +5132,15 @@
         <v>1.5</v>
       </c>
       <c r="G125" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="H125" s="2" t="n">
+      <c r="I125" s="2" t="n">
         <v>10.8</v>
       </c>
-      <c r="I125" s="2" t="inlineStr">
+      <c r="J125" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -4794,12 +5172,15 @@
         <v>2</v>
       </c>
       <c r="G126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H126" s="2" t="n">
+      <c r="I126" s="2" t="n">
         <v>5.3</v>
       </c>
-      <c r="I126" s="2" t="inlineStr">
+      <c r="J126" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -4831,12 +5212,15 @@
         <v>0</v>
       </c>
       <c r="G127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="H127" s="2" t="n">
+      <c r="I127" s="2" t="n">
         <v>5.3</v>
       </c>
-      <c r="I127" s="2" t="inlineStr">
+      <c r="J127" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -4868,12 +5252,15 @@
         <v>1.5</v>
       </c>
       <c r="G128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="H128" s="2" t="n">
+      <c r="I128" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I128" s="2" t="inlineStr">
+      <c r="J128" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -4905,12 +5292,15 @@
         <v>-1.5</v>
       </c>
       <c r="G129" s="2" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="H129" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="H129" s="2" t="n">
+      <c r="I129" s="2" t="n">
         <v>5.4</v>
       </c>
-      <c r="I129" s="2" t="inlineStr">
+      <c r="J129" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -4942,12 +5332,15 @@
         <v>-2.5</v>
       </c>
       <c r="G130" s="2" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="H130" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="H130" s="2" t="n">
+      <c r="I130" s="2" t="n">
         <v>7.8</v>
       </c>
-      <c r="I130" s="2" t="inlineStr"/>
+      <c r="J130" s="2" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -4975,12 +5368,15 @@
         <v>-1</v>
       </c>
       <c r="G131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="H131" s="2" t="n">
+      <c r="I131" s="2" t="n">
         <v>12.3</v>
       </c>
-      <c r="I131" s="2" t="inlineStr">
+      <c r="J131" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5012,12 +5408,15 @@
         <v>0.5</v>
       </c>
       <c r="G132" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H132" s="2" t="n">
+      <c r="I132" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="I132" s="2" t="inlineStr">
+      <c r="J132" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5049,12 +5448,15 @@
         <v>1</v>
       </c>
       <c r="G133" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H133" s="2" t="n">
+      <c r="I133" s="2" t="n">
         <v>2.2</v>
       </c>
-      <c r="I133" s="2" t="inlineStr">
+      <c r="J133" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5086,12 +5488,15 @@
         <v>-0.5</v>
       </c>
       <c r="G134" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H134" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H134" s="2" t="n">
+      <c r="I134" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I134" s="2" t="inlineStr">
+      <c r="J134" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5123,12 +5528,15 @@
         <v>-0.5</v>
       </c>
       <c r="G135" s="2" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="H135" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H135" s="2" t="n">
+      <c r="I135" s="2" t="n">
         <v>3.3</v>
       </c>
-      <c r="I135" s="2" t="inlineStr"/>
+      <c r="J135" s="2" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -5156,12 +5564,15 @@
         <v>-1</v>
       </c>
       <c r="G136" s="2" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="H136" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H136" s="2" t="n">
+      <c r="I136" s="2" t="n">
         <v>8.1</v>
       </c>
-      <c r="I136" s="2" t="inlineStr"/>
+      <c r="J136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -5189,12 +5600,15 @@
         <v>0.5</v>
       </c>
       <c r="G137" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H137" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="H137" s="2" t="n">
+      <c r="I137" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I137" s="2" t="inlineStr"/>
+      <c r="J137" s="2" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -5222,12 +5636,15 @@
         <v>0.5</v>
       </c>
       <c r="G138" s="2" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="H138" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H138" s="2" t="n">
+      <c r="I138" s="2" t="n">
         <v>11.2</v>
       </c>
-      <c r="I138" s="2" t="inlineStr"/>
+      <c r="J138" s="2" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -5255,12 +5672,15 @@
         <v>1.5</v>
       </c>
       <c r="G139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H139" s="2" t="n">
+      <c r="I139" s="2" t="n">
         <v>5.9</v>
       </c>
-      <c r="I139" s="2" t="inlineStr">
+      <c r="J139" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5292,12 +5712,15 @@
         <v>0.5</v>
       </c>
       <c r="G140" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H140" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="H140" s="2" t="n">
+      <c r="I140" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="I140" s="2" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -5325,12 +5748,15 @@
         <v>0.5</v>
       </c>
       <c r="G141" s="2" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="H141" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="H141" s="2" t="n">
+      <c r="I141" s="2" t="n">
         <v>11.3</v>
       </c>
-      <c r="I141" s="2" t="inlineStr"/>
+      <c r="J141" s="2" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -5358,12 +5784,15 @@
         <v>-1.5</v>
       </c>
       <c r="G142" s="2" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="H142" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H142" s="2" t="n">
+      <c r="I142" s="2" t="n">
         <v>2.8</v>
       </c>
-      <c r="I142" s="2" t="inlineStr">
+      <c r="J142" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -5395,12 +5824,15 @@
         <v>-1</v>
       </c>
       <c r="G143" s="2" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="H143" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="H143" s="2" t="n">
+      <c r="I143" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="I143" s="2" t="inlineStr"/>
+      <c r="J143" s="2" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -5428,12 +5860,15 @@
         <v>-4</v>
       </c>
       <c r="G144" s="2" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="H144" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H144" s="2" t="n">
+      <c r="I144" s="2" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="I144" s="2" t="inlineStr"/>
+      <c r="J144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -5461,12 +5896,15 @@
         <v>0</v>
       </c>
       <c r="G145" s="2" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="H145" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H145" s="2" t="n">
+      <c r="I145" s="2" t="n">
         <v>4.7</v>
       </c>
-      <c r="I145" s="2" t="inlineStr"/>
+      <c r="J145" s="2" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -5494,12 +5932,15 @@
         <v>0.5</v>
       </c>
       <c r="G146" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="H146" s="2" t="n">
+      <c r="I146" s="2" t="n">
         <v>9.1</v>
       </c>
-      <c r="I146" s="2" t="inlineStr">
+      <c r="J146" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5531,12 +5972,15 @@
         <v>-2</v>
       </c>
       <c r="G147" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="H147" s="2" t="n">
+      <c r="I147" s="2" t="n">
         <v>1.2</v>
       </c>
-      <c r="I147" s="2" t="inlineStr">
+      <c r="J147" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5568,12 +6012,15 @@
         <v>-2</v>
       </c>
       <c r="G148" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="H148" s="2" t="n">
+      <c r="I148" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="I148" s="2" t="inlineStr">
+      <c r="J148" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5605,12 +6052,15 @@
         <v>-4</v>
       </c>
       <c r="G149" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="H149" s="2" t="n">
+      <c r="I149" s="2" t="n">
         <v>2.9</v>
       </c>
-      <c r="I149" s="2" t="inlineStr">
+      <c r="J149" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5642,12 +6092,15 @@
         <v>1</v>
       </c>
       <c r="G150" s="2" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="H150" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="H150" s="2" t="n">
+      <c r="I150" s="2" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="I150" s="2" t="inlineStr">
+      <c r="J150" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -5679,12 +6132,15 @@
         <v>0.5</v>
       </c>
       <c r="G151" s="2" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="H151" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="H151" s="2" t="n">
+      <c r="I151" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="I151" s="2" t="inlineStr"/>
+      <c r="J151" s="2" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -5712,12 +6168,15 @@
         <v>-0.5</v>
       </c>
       <c r="G152" s="2" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="H152" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="H152" s="2" t="n">
+      <c r="I152" s="2" t="n">
         <v>13.3</v>
       </c>
-      <c r="I152" s="2" t="inlineStr"/>
+      <c r="J152" s="2" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -5745,12 +6204,15 @@
         <v>-1</v>
       </c>
       <c r="G153" s="2" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="H153" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="H153" s="2" t="n">
+      <c r="I153" s="2" t="n">
         <v>15.3</v>
       </c>
-      <c r="I153" s="2" t="inlineStr"/>
+      <c r="J153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -5778,12 +6240,15 @@
         <v>0</v>
       </c>
       <c r="G154" s="2" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="H154" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H154" s="2" t="n">
+      <c r="I154" s="2" t="n">
         <v>7.7</v>
       </c>
-      <c r="I154" s="2" t="inlineStr"/>
+      <c r="J154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -5811,12 +6276,15 @@
         <v>0.5</v>
       </c>
       <c r="G155" s="2" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="H155" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H155" s="2" t="n">
+      <c r="I155" s="2" t="n">
         <v>1.9</v>
       </c>
-      <c r="I155" s="2" t="inlineStr"/>
+      <c r="J155" s="2" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -5844,12 +6312,15 @@
         <v>0</v>
       </c>
       <c r="G156" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="H156" s="2" t="n">
+      <c r="I156" s="2" t="n">
         <v>2.4</v>
       </c>
-      <c r="I156" s="2" t="inlineStr">
+      <c r="J156" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -5881,12 +6352,15 @@
         <v>-1.5</v>
       </c>
       <c r="G157" s="2" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="H157" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="H157" s="2" t="n">
+      <c r="I157" s="2" t="n">
         <v>9.4</v>
       </c>
-      <c r="I157" s="2" t="inlineStr"/>
+      <c r="J157" s="2" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -5914,12 +6388,15 @@
         <v>-2.5</v>
       </c>
       <c r="G158" s="2" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="H158" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H158" s="2" t="n">
+      <c r="I158" s="2" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="I158" s="2" t="inlineStr">
+      <c r="J158" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -5951,12 +6428,15 @@
         <v>-3.5</v>
       </c>
       <c r="G159" s="2" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="H159" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H159" s="2" t="n">
+      <c r="I159" s="2" t="n">
         <v>6.5</v>
       </c>
-      <c r="I159" s="2" t="inlineStr">
+      <c r="J159" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -5988,12 +6468,15 @@
         <v>0</v>
       </c>
       <c r="G160" s="2" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="H160" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H160" s="2" t="n">
+      <c r="I160" s="2" t="n">
         <v>9.5</v>
       </c>
-      <c r="I160" s="2" t="inlineStr"/>
+      <c r="J160" s="2" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -6021,12 +6504,15 @@
         <v>-1</v>
       </c>
       <c r="G161" s="2" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H161" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="H161" s="2" t="n">
+      <c r="I161" s="2" t="n">
         <v>10.7</v>
       </c>
-      <c r="I161" s="2" t="inlineStr"/>
+      <c r="J161" s="2" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -6054,12 +6540,15 @@
         <v>-1</v>
       </c>
       <c r="G162" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H162" s="2" t="n">
+      <c r="I162" s="2" t="n">
         <v>24.8</v>
       </c>
-      <c r="I162" s="2" t="inlineStr">
+      <c r="J162" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -6091,12 +6580,15 @@
         <v>-1</v>
       </c>
       <c r="G163" s="2" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="H163" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="H163" s="2" t="n">
+      <c r="I163" s="2" t="n">
         <v>66.90000000000001</v>
       </c>
-      <c r="I163" s="2" t="inlineStr"/>
+      <c r="J163" s="2" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -6124,12 +6616,15 @@
         <v>-1.5</v>
       </c>
       <c r="G164" s="2" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="H164" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="H164" s="2" t="n">
+      <c r="I164" s="2" t="n">
         <v>8.9</v>
       </c>
-      <c r="I164" s="2" t="inlineStr"/>
+      <c r="J164" s="2" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -6157,12 +6652,15 @@
         <v>-1.5</v>
       </c>
       <c r="G165" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H165" s="2" t="n">
+      <c r="I165" s="2" t="n">
         <v>2.7</v>
       </c>
-      <c r="I165" s="2" t="inlineStr">
+      <c r="J165" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -6194,12 +6692,15 @@
         <v>-0.5</v>
       </c>
       <c r="G166" s="2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="H166" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H166" s="2" t="n">
+      <c r="I166" s="2" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="I166" s="2" t="inlineStr"/>
+      <c r="J166" s="2" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -6227,12 +6728,15 @@
         <v>-1.5</v>
       </c>
       <c r="G167" s="2" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="H167" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H167" s="2" t="n">
+      <c r="I167" s="2" t="n">
         <v>3.7</v>
       </c>
-      <c r="I167" s="2" t="inlineStr">
+      <c r="J167" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -6264,12 +6768,15 @@
         <v>-5</v>
       </c>
       <c r="G168" s="2" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="H168" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H168" s="2" t="n">
+      <c r="I168" s="2" t="n">
         <v>4.3</v>
       </c>
-      <c r="I168" s="2" t="inlineStr">
+      <c r="J168" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY</t>
         </is>
@@ -6301,12 +6808,15 @@
         <v>-5</v>
       </c>
       <c r="G169" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H169" s="2" t="n">
+      <c r="I169" s="2" t="n">
         <v>11.6</v>
       </c>
-      <c r="I169" s="2" t="inlineStr">
+      <c r="J169" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -6338,12 +6848,15 @@
         <v>-4.5</v>
       </c>
       <c r="G170" s="2" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="H170" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H170" s="2" t="n">
+      <c r="I170" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="I170" s="2" t="inlineStr">
+      <c r="J170" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -6375,12 +6888,15 @@
         <v>-4</v>
       </c>
       <c r="G171" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H171" s="2" t="n">
+      <c r="I171" s="2" t="n">
         <v>3.2</v>
       </c>
-      <c r="I171" s="2" t="inlineStr">
+      <c r="J171" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -6412,12 +6928,15 @@
         <v>-3.5</v>
       </c>
       <c r="G172" s="2" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="H172" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="H172" s="2" t="n">
+      <c r="I172" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="I172" s="2" t="inlineStr"/>
+      <c r="J172" s="2" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -6445,12 +6964,15 @@
         <v>-3</v>
       </c>
       <c r="G173" s="2" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="H173" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H173" s="2" t="n">
+      <c r="I173" s="2" t="n">
         <v>4.2</v>
       </c>
-      <c r="I173" s="2" t="inlineStr"/>
+      <c r="J173" s="2" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -6478,12 +7000,15 @@
         <v>0</v>
       </c>
       <c r="G174" s="2" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="H174" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="H174" s="2" t="n">
+      <c r="I174" s="2" t="n">
         <v>60.6</v>
       </c>
-      <c r="I174" s="2" t="inlineStr"/>
+      <c r="J174" s="2" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -6511,12 +7036,15 @@
         <v>-2</v>
       </c>
       <c r="G175" s="2" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="H175" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H175" s="2" t="n">
+      <c r="I175" s="2" t="n">
         <v>2.8</v>
       </c>
-      <c r="I175" s="2" t="inlineStr"/>
+      <c r="J175" s="2" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -6544,12 +7072,15 @@
         <v>-3</v>
       </c>
       <c r="G176" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="H176" s="2" t="n">
+      <c r="I176" s="2" t="n">
         <v>2.4</v>
       </c>
-      <c r="I176" s="2" t="inlineStr">
+      <c r="J176" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -6581,12 +7112,15 @@
         <v>-1.5</v>
       </c>
       <c r="G177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="H177" s="2" t="n">
+      <c r="I177" s="2" t="n">
         <v>6.1</v>
       </c>
-      <c r="I177" s="2" t="inlineStr">
+      <c r="J177" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -6618,12 +7152,15 @@
         <v>-1.5</v>
       </c>
       <c r="G178" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H178" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="H178" s="2" t="n">
+      <c r="I178" s="2" t="n">
         <v>17.7</v>
       </c>
-      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -6651,12 +7188,15 @@
         <v>-4.5</v>
       </c>
       <c r="G179" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H179" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="H179" s="2" t="n">
+      <c r="I179" s="2" t="n">
         <v>5.8</v>
       </c>
-      <c r="I179" s="2" t="inlineStr">
+      <c r="J179" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -6688,12 +7228,15 @@
         <v>-1.5</v>
       </c>
       <c r="G180" s="2" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="H180" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H180" s="2" t="n">
+      <c r="I180" s="2" t="n">
         <v>6.5</v>
       </c>
-      <c r="I180" s="2" t="inlineStr"/>
+      <c r="J180" s="2" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -6721,12 +7264,15 @@
         <v>0</v>
       </c>
       <c r="G181" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H181" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H181" s="2" t="n">
+      <c r="I181" s="2" t="n">
         <v>21.9</v>
       </c>
-      <c r="I181" s="2" t="inlineStr">
+      <c r="J181" s="2" t="inlineStr">
         <is>
           <t>HIGH UNCERTAINTY - MANUAL REVIEW NEEDED</t>
         </is>
@@ -6743,17 +7289,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6769,6 +7316,7 @@
       <c r="F1" s="6" t="n"/>
       <c r="G1" s="6" t="n"/>
       <c r="H1" s="6" t="n"/>
+      <c r="I1" s="6" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -6783,30 +7331,35 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>VP</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Expected Best-3</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Actual Best-3</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>IGL</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>Transfers</t>
         </is>
@@ -6825,100 +7378,120 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>I</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="E3" s="2" t="n">
         <v>7.5</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="F3" s="2" t="n">
         <v>30.2</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MaKo</t>
+          <t>JohnQT</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>DRX</t>
+          <t>Sentinels</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>8.5</v>
-      </c>
       <c r="E4" s="2" t="n">
-        <v>35.7</v>
+        <v>7.5</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+        <v>28.7</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>SociablEE</t>
+          <t>Free1ng</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Natus Vincere</t>
+          <t>DRX</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E5" s="2" t="n">
-        <v>34.1</v>
-      </c>
       <c r="F5" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
+        <v>34.8</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Free1ng</t>
+          <t>skuba</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>DRX</t>
+          <t>NRG Esports</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>S</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>8</v>
-      </c>
       <c r="E6" s="2" t="n">
-        <v>34.9</v>
+        <v>9.5</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+        <v>38.9</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -6933,51 +7506,61 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>S</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="E7" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="E7" s="2" t="n">
-        <v>35.6</v>
-      </c>
       <c r="F7" s="2" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>brawk</t>
+          <t>Karon</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>NRG Esports</t>
+          <t>Gen.G</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>10.5</v>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>44</v>
+        <v>9.5</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+        <v>35.8</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>skuba</t>
+          <t>brawk</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -6987,73 +7570,88 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>9.5</v>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>38.9</v>
+        <v>10.5</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
+        <v>43.8</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>JohnQT</t>
+          <t>SociablEE</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Sentinels</t>
+          <t>Natus Vincere</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>7.5</v>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>28.7</v>
+        <v>8</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
+        <v>34.3</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PROFEK</t>
+          <t>MaKo</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Team Vitality</t>
+          <t>DRX</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
-        <v>9</v>
-      </c>
       <c r="E11" s="2" t="n">
-        <v>32.8</v>
+        <v>8.5</v>
       </c>
       <c r="F11" s="2" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -7068,19 +7666,24 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="E12" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E12" s="2" t="n">
-        <v>50.5</v>
-      </c>
       <c r="F12" s="2" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>IGL</t>
         </is>
@@ -7099,19 +7702,24 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
           <t>D</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="E13" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="F13" s="2" t="n">
         <v>33.2</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -7119,14 +7727,14 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
-        <v>99.5</v>
-      </c>
       <c r="E14" s="9" t="n">
-        <v>449.2</v>
-      </c>
-      <c r="F14" s="10" t="n">
-        <v>305</v>
+        <v>100</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>451.8</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>